<commit_message>
Versión final del proyecto terminada
</commit_message>
<xml_diff>
--- a/BackEnd/Excels/Asistencias_totales.xlsx
+++ b/BackEnd/Excels/Asistencias_totales.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josue\Downloads\Formatos excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josue\Programacion\HerramientaDeServicio-main (1)\HerramientaDeServicio-main\BackEnd\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{466D688C-4EAB-4FBA-9937-7483C73A2B16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB7FF01-26AB-4DA2-B512-CC3FC5C88C24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{282BC857-CBD7-44D5-8295-81F2ADA10FD4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="18">
   <si>
     <t>V</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Fecha</t>
-  </si>
-  <si>
     <t>Dia</t>
   </si>
   <si>
@@ -78,13 +75,31 @@
   </si>
   <si>
     <t>Seccion:</t>
+  </si>
+  <si>
+    <t>Semanas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lunes </t>
+  </si>
+  <si>
+    <t>Martes</t>
+  </si>
+  <si>
+    <t>Miercoles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jueves </t>
+  </si>
+  <si>
+    <t>Viernes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -118,16 +133,30 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -150,41 +179,344 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -526,22 +858,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-    </row>
-    <row r="2" spans="1:10" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A1" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+    </row>
+    <row r="2" spans="1:10" ht="26.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>0</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -552,99 +884,119 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="G3" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
+      <c r="A3" s="17">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+      <c r="G3" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
     </row>
     <row r="4" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
+      <c r="A4" s="18"/>
+      <c r="B4" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
+      <c r="E4" s="10"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
     </row>
     <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
+      <c r="A5" s="18"/>
+      <c r="B5" s="9" t="s">
+        <v>15</v>
+      </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="G5" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="H5" s="5" t="s">
+      <c r="E5" s="10"/>
+      <c r="G5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
+      <c r="A6" s="18"/>
+      <c r="B6" s="9" t="s">
+        <v>16</v>
+      </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
+      <c r="E6" s="10"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
+    <row r="7" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="19"/>
+      <c r="B7" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="13"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
+      <c r="A8" s="20">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="8"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
+      <c r="E9" s="10"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
+      <c r="A10" s="18"/>
+      <c r="B10" s="9" t="s">
+        <v>15</v>
+      </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="G10" s="10" t="s">
+      <c r="E10" s="10"/>
+      <c r="G10" s="3" t="s">
         <v>2</v>
       </c>
       <c r="H10" s="1"/>
@@ -652,153 +1004,167 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="9" t="s">
+        <v>16</v>
+      </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
+      <c r="E11" s="10"/>
+    </row>
+    <row r="12" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="19"/>
+      <c r="B12" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="13"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
+      <c r="A13" s="20">
+        <v>3</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="G14" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="H14" s="11"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
+      <c r="E14" s="10"/>
+      <c r="G14" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="25"/>
+      <c r="I14" s="26"/>
+      <c r="J14" s="27"/>
     </row>
     <row r="15" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="9" t="s">
+        <v>15</v>
+      </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="G15" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="H15" s="11"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
+      <c r="E15" s="10"/>
+      <c r="G15" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="24"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="29"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="9" t="s">
+        <v>16</v>
+      </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
+      <c r="E16" s="10"/>
+    </row>
+    <row r="17" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="19"/>
+      <c r="B17" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="13"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
+      <c r="A18" s="20">
+        <v>4</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="8"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
+      <c r="E19" s="10"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="9" t="s">
+        <v>15</v>
+      </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
+      <c r="E20" s="10"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="9" t="s">
+        <v>16</v>
+      </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
+      <c r="E21" s="10"/>
+    </row>
+    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="21"/>
+      <c r="B22" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="13"/>
     </row>
     <row r="23" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" s="23"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+    </row>
+    <row r="24" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-    </row>
-    <row r="24" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B24" s="2"/>
+      <c r="B24" s="14"/>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
     </row>
     <row r="25" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" s="2"/>
+      <c r="A25" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" s="14"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="G3:J4"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G14:H14"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="A13:A17"/>
+    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>